<commit_message>
Changes when working to extend the range.
</commit_message>
<xml_diff>
--- a/hodor/Wemos Board Pinning.xlsx
+++ b/hodor/Wemos Board Pinning.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="18201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="18431"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="46">
   <si>
     <t>Board Pin</t>
   </si>
@@ -159,6 +159,9 @@
   </si>
   <si>
     <t>do not use this pin</t>
+  </si>
+  <si>
+    <t>Board programming:</t>
   </si>
 </sst>
 </file>
@@ -270,15 +273,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
-      <xdr:row>16</xdr:row>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>238125</xdr:colOff>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>180975</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>3713995</xdr:colOff>
-      <xdr:row>34</xdr:row>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>189745</xdr:colOff>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>75784</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -302,8 +305,52 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5905500" y="3219450"/>
+          <a:off x="8467725" y="3409950"/>
           <a:ext cx="6038095" cy="3323809"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>9923</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>133923</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9388B9EB-E530-403F-B191-C96F611EC886}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5391150" y="3448050"/>
+          <a:ext cx="2848373" cy="4105848"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -850,7 +897,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B17" s="10" t="s">
         <v>33</v>
       </c>
@@ -861,7 +908,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B18" s="10" t="s">
         <v>33</v>
       </c>
@@ -871,8 +918,11 @@
       <c r="D18" s="10" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>11</v>
       </c>
@@ -885,8 +935,9 @@
       <c r="D19" s="10" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F19" s="10"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B20" s="10" t="s">
         <v>33</v>
       </c>
@@ -897,7 +948,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="10" t="s">
         <v>33</v>

</xml_diff>